<commit_message>
tests from R and scipy used to improve Stats::LikeR
</commit_message>
<xml_diff>
--- a/lang.compare.xlsx
+++ b/lang.compare.xlsx
@@ -74,19 +74,19 @@
         </is>
       </c>
       <c r="B2">
-        <v>2.74470610472921e-06</v>
+        <v>3.87821087088902e-06</v>
       </c>
       <c r="C2">
-        <v>0.000157445037725016</v>
+        <v>0.0001505990185251</v>
       </c>
       <c r="D2">
-        <v>7.93252672467914e-05</v>
+        <v>7.24792480468751e-05</v>
       </c>
       <c r="E2">
-        <v>0.000106573104858398</v>
+        <v>0.000113419124058315</v>
       </c>
       <c r="F2">
-        <v>-0.000157445037725016</v>
+        <v>-0.0001505990185251</v>
       </c>
       <c r="G2">
         <v>-7.81197704782244e-05</v>
@@ -95,7 +95,7 @@
         <v>0.000264018142583414</v>
       </c>
       <c r="I2">
-        <v>-7.93252672467914e-05</v>
+        <v>-7.24792480468751e-05</v>
       </c>
       <c r="J2">
         <v>7.81197704782244e-05</v>
@@ -111,19 +111,19 @@
         </is>
       </c>
       <c r="B3">
-        <v>2.08273507329437e-08</v>
+        <v>0.819443099233151</v>
       </c>
       <c r="C3">
-        <v>-0.00158128706711328</v>
+        <v>1.43764035393738e-06</v>
       </c>
       <c r="D3">
-        <v>-0.00165299006870815</v>
+        <v>-7.02653612409322e-05</v>
       </c>
       <c r="E3">
-        <v>0.00197928292410714</v>
+        <v>0.000396558216639928</v>
       </c>
       <c r="F3">
-        <v>0.00158128706711328</v>
+        <v>-1.43764035393738e-06</v>
       </c>
       <c r="G3">
         <v>-7.17030015948696e-05</v>
@@ -132,7 +132,7 @@
         <v>0.000397995856993865</v>
       </c>
       <c r="I3">
-        <v>0.00165299006870815</v>
+        <v>7.02653612409322e-05</v>
       </c>
       <c r="J3">
         <v>7.17030015948696e-05</v>
@@ -148,19 +148,19 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.000517946020100579</v>
+        <v>0.00181238974913112</v>
       </c>
       <c r="C4">
-        <v>0.000156729064786175</v>
+        <v>0.000129685585956655</v>
       </c>
       <c r="D4">
-        <v>1.21593475341795e-05</v>
+        <v>-1.48841312953404e-05</v>
       </c>
       <c r="E4">
-        <v>0.000180278505597796</v>
+        <v>0.000207321984427316</v>
       </c>
       <c r="F4">
-        <v>-0.000156729064786175</v>
+        <v>-0.000129685585956655</v>
       </c>
       <c r="G4">
         <v>-0.000144569717251995</v>
@@ -169,7 +169,7 @@
         <v>0.00033700757038397</v>
       </c>
       <c r="I4">
-        <v>-1.21593475341795e-05</v>
+        <v>1.48841312953404e-05</v>
       </c>
       <c r="J4">
         <v>0.000144569717251995</v>
@@ -185,19 +185,19 @@
         </is>
       </c>
       <c r="B5">
-        <v>3.63139969150605e-05</v>
+        <v>0.000272825863196768</v>
       </c>
       <c r="C5">
-        <v>0.000126131723975829</v>
+        <v>0.000100893414388078</v>
       </c>
       <c r="D5">
-        <v>1.91756657191685e-05</v>
+        <v>-6.06264386858254e-06</v>
       </c>
       <c r="E5">
-        <v>0.000176974705287388</v>
+        <v>0.000202213014875139</v>
       </c>
       <c r="F5">
-        <v>-0.000126131723975829</v>
+        <v>-0.000100893414388078</v>
       </c>
       <c r="G5">
         <v>-0.000106956058256661</v>
@@ -206,7 +206,7 @@
         <v>0.000303106429263218</v>
       </c>
       <c r="I5">
-        <v>-1.91756657191685e-05</v>
+        <v>6.06264386858254e-06</v>
       </c>
       <c r="J5">
         <v>0.000106956058256661</v>
@@ -222,19 +222,19 @@
         </is>
       </c>
       <c r="B6">
-        <v>7.79914130610848e-07</v>
+        <v>1.77722144423242e-06</v>
       </c>
       <c r="C6">
-        <v>0.000137633565567999</v>
+        <v>0.00011951375355628</v>
       </c>
       <c r="D6">
-        <v>2.81333923339845e-05</v>
+        <v>1.00135803222654e-05</v>
       </c>
       <c r="E6">
-        <v>0.000124011720929827</v>
+        <v>0.000142131532941546</v>
       </c>
       <c r="F6">
-        <v>-0.000137633565567999</v>
+        <v>-0.00011951375355628</v>
       </c>
       <c r="G6">
         <v>-0.000109500173234015</v>
@@ -243,7 +243,7 @@
         <v>0.000261645286497826</v>
       </c>
       <c r="I6">
-        <v>-2.81333923339845e-05</v>
+        <v>-1.00135803222654e-05</v>
       </c>
       <c r="J6">
         <v>0.000109500173234015</v>
@@ -259,19 +259,19 @@
         </is>
       </c>
       <c r="B7">
-        <v>7.0791270745385e-07</v>
+        <v>1.09246928370332e-06</v>
       </c>
       <c r="C7">
-        <v>0.00010975116726643</v>
+        <v>9.67743846039023e-05</v>
       </c>
       <c r="D7">
-        <v>1.41348157610212e-05</v>
+        <v>1.15803309849339e-06</v>
       </c>
       <c r="E7">
-        <v>0.000130585261753627</v>
+        <v>0.000143562044416155</v>
       </c>
       <c r="F7">
-        <v>-0.00010975116726643</v>
+        <v>-9.67743846039023e-05</v>
       </c>
       <c r="G7">
         <v>-9.56163515054089e-05</v>
@@ -280,7 +280,7 @@
         <v>0.000240336429020057</v>
       </c>
       <c r="I7">
-        <v>-1.41348157610212e-05</v>
+        <v>-1.15803309849339e-06</v>
       </c>
       <c r="J7">
         <v>9.56163515054089e-05</v>
@@ -296,19 +296,19 @@
         </is>
       </c>
       <c r="B8">
-        <v>7.28950727113542e-07</v>
+        <v>2.54653950815253e-07</v>
       </c>
       <c r="C8">
-        <v>-0.00112013103301121</v>
+        <v>-0.00126941512332581</v>
       </c>
       <c r="D8">
-        <v>-0.00113926615033831</v>
+        <v>-0.0012885502406529</v>
       </c>
       <c r="E8">
-        <v>0.00179699489048549</v>
+        <v>0.00194627898080008</v>
       </c>
       <c r="F8">
-        <v>0.00112013103301121</v>
+        <v>0.00126941512332581</v>
       </c>
       <c r="G8">
         <v>-1.91351173270965e-05</v>
@@ -317,7 +317,7 @@
         <v>0.000676863857474278</v>
       </c>
       <c r="I8">
-        <v>0.00113926615033831</v>
+        <v>0.0012885502406529</v>
       </c>
       <c r="J8">
         <v>1.91351173270965e-05</v>
@@ -333,19 +333,19 @@
         </is>
       </c>
       <c r="B9">
-        <v>0.0106364440002353</v>
+        <v>0.00958849120382088</v>
       </c>
       <c r="C9">
-        <v>8.02352936131816e-05</v>
+        <v>9.32461360727237e-05</v>
       </c>
       <c r="D9">
-        <v>-0.000166927065168109</v>
+        <v>-0.000153916222708566</v>
       </c>
       <c r="E9">
-        <v>0.000481298991612025</v>
+        <v>0.000468288149152483</v>
       </c>
       <c r="F9">
-        <v>-8.02352936131816e-05</v>
+        <v>-9.32461360727237e-05</v>
       </c>
       <c r="G9">
         <v>-0.00024716235878129</v>
@@ -354,7 +354,7 @@
         <v>0.000561534285225207</v>
       </c>
       <c r="I9">
-        <v>0.000166927065168109</v>
+        <v>0.000153916222708566</v>
       </c>
       <c r="J9">
         <v>0.00024716235878129</v>
@@ -370,19 +370,19 @@
         </is>
       </c>
       <c r="B10">
-        <v>1.53044625831322e-05</v>
+        <v>1.41446033696813e-06</v>
       </c>
       <c r="C10">
-        <v>-0.000112551819516479</v>
+        <v>-0.000127333771420776</v>
       </c>
       <c r="D10">
-        <v>-0.000263588769095284</v>
+        <v>-0.000278370720999581</v>
       </c>
       <c r="E10">
-        <v>0.000532627105712891</v>
+        <v>0.000547409057617187</v>
       </c>
       <c r="F10">
-        <v>0.000112551819516479</v>
+        <v>0.000127333771420776</v>
       </c>
       <c r="G10">
         <v>-0.000151036949578805</v>
@@ -391,7 +391,7 @@
         <v>0.000420075286196412</v>
       </c>
       <c r="I10">
-        <v>0.000263588769095284</v>
+        <v>0.000278370720999581</v>
       </c>
       <c r="J10">
         <v>0.000151036949578805</v>
@@ -407,19 +407,19 @@
         </is>
       </c>
       <c r="B11">
-        <v>8.54804951266885e-08</v>
+        <v>8.59630733263117e-09</v>
       </c>
       <c r="C11">
-        <v>-0.000123782268409351</v>
+        <v>-0.000125314959275004</v>
       </c>
       <c r="D11">
-        <v>-2.40462166922433e-05</v>
+        <v>-2.55789075578961e-05</v>
       </c>
       <c r="E11">
-        <v>0.000159638268607003</v>
+        <v>0.000161170959472656</v>
       </c>
       <c r="F11">
-        <v>0.000123782268409351</v>
+        <v>0.000125314959275004</v>
       </c>
       <c r="G11">
         <v>9.97360517171078e-05</v>
@@ -428,7 +428,7 @@
         <v>3.58560001976522e-05</v>
       </c>
       <c r="I11">
-        <v>2.40462166922433e-05</v>
+        <v>2.55789075578961e-05</v>
       </c>
       <c r="J11">
         <v>-9.97360517171078e-05</v>
@@ -444,19 +444,19 @@
         </is>
       </c>
       <c r="B12">
-        <v>4.45505047297345e-08</v>
+        <v>2.77440471707635e-08</v>
       </c>
       <c r="C12">
-        <v>-0.000103808798095477</v>
+        <v>-0.000112085328770003</v>
       </c>
       <c r="D12">
-        <v>-1.10353742327008e-05</v>
+        <v>-1.93119049072267e-05</v>
       </c>
       <c r="E12">
-        <v>0.000127553939819336</v>
+        <v>0.000135830470493862</v>
       </c>
       <c r="F12">
-        <v>0.000103808798095477</v>
+        <v>0.000112085328770003</v>
       </c>
       <c r="G12">
         <v>9.27734238627766e-05</v>
@@ -465,7 +465,7 @@
         <v>2.37451417238585e-05</v>
       </c>
       <c r="I12">
-        <v>1.10353742327008e-05</v>
+        <v>1.93119049072267e-05</v>
       </c>
       <c r="J12">
         <v>-9.27734238627766e-05</v>
@@ -481,19 +481,19 @@
         </is>
       </c>
       <c r="B13">
-        <v>2.94921223198408e-06</v>
+        <v>2.28701351423499e-06</v>
       </c>
       <c r="C13">
-        <v>-0.00235668604831777</v>
+        <v>-0.00253836100559316</v>
       </c>
       <c r="D13">
-        <v>-0.00359211649213518</v>
+        <v>-0.00377379144941057</v>
       </c>
       <c r="E13">
-        <v>0.00518574033464704</v>
+        <v>0.00536741529192243</v>
       </c>
       <c r="F13">
-        <v>0.00235668604831777</v>
+        <v>0.00253836100559316</v>
       </c>
       <c r="G13">
         <v>-0.00123543044381742</v>
@@ -502,7 +502,7 @@
         <v>0.00282905428632928</v>
       </c>
       <c r="I13">
-        <v>0.00359211649213518</v>
+        <v>0.00377379144941057</v>
       </c>
       <c r="J13">
         <v>0.00123543044381742</v>
@@ -518,19 +518,19 @@
         </is>
       </c>
       <c r="B14">
-        <v>4.77728967496205e-13</v>
+        <v>4.2765790908561e-13</v>
       </c>
       <c r="C14">
-        <v>-0.00389312765556887</v>
+        <v>-0.00399844054793773</v>
       </c>
       <c r="D14">
-        <v>0.00446724891662595</v>
+        <v>0.00436193602425709</v>
       </c>
       <c r="E14">
-        <v>0.00746965408325195</v>
+        <v>0.00757496697562081</v>
       </c>
       <c r="F14">
-        <v>0.00389312765556887</v>
+        <v>0.00399844054793773</v>
       </c>
       <c r="G14">
         <v>0.00836037657219481</v>
@@ -539,7 +539,7 @@
         <v>0.00357652642768309</v>
       </c>
       <c r="I14">
-        <v>-0.00446724891662595</v>
+        <v>-0.00436193602425709</v>
       </c>
       <c r="J14">
         <v>-0.00836037657219481</v>
@@ -555,19 +555,19 @@
         </is>
       </c>
       <c r="B15">
-        <v>9.74480385274035e-10</v>
+        <v>8.95056251337678e-11</v>
       </c>
       <c r="C15">
-        <v>-0.0101350002862871</v>
+        <v>-0.0108087371310311</v>
       </c>
       <c r="D15">
-        <v>-0.0149615492139544</v>
+        <v>-0.0156352860586984</v>
       </c>
       <c r="E15">
-        <v>0.0162365777151925</v>
+        <v>0.0169103145599365</v>
       </c>
       <c r="F15">
-        <v>0.0101350002862871</v>
+        <v>0.0108087371310311</v>
       </c>
       <c r="G15">
         <v>-0.00482654892766732</v>
@@ -576,7 +576,7 @@
         <v>0.00610157742890546</v>
       </c>
       <c r="I15">
-        <v>0.0149615492139544</v>
+        <v>0.0156352860586984</v>
       </c>
       <c r="J15">
         <v>0.00482654892766732</v>
@@ -592,19 +592,19 @@
         </is>
       </c>
       <c r="B16">
-        <v>1.21929841778723e-08</v>
+        <v>4.37108660888974e-06</v>
       </c>
       <c r="C16">
-        <v>-0.000763176494988979</v>
+        <v>-0.000825437803931499</v>
       </c>
       <c r="D16">
-        <v>-0.000811917441231864</v>
+        <v>-0.000874178750174384</v>
       </c>
       <c r="E16">
-        <v>0.00142124720982143</v>
+        <v>0.00148350851876395</v>
       </c>
       <c r="F16">
-        <v>0.000763176494988979</v>
+        <v>0.000825437803931499</v>
       </c>
       <c r="G16">
         <v>-4.87409462428857e-05</v>
@@ -613,7 +613,7 @@
         <v>0.00065807071483245</v>
       </c>
       <c r="I16">
-        <v>0.000811917441231864</v>
+        <v>0.000874178750174384</v>
       </c>
       <c r="J16">
         <v>4.87409462428857e-05</v>
@@ -629,19 +629,19 @@
         </is>
       </c>
       <c r="B17">
-        <v>0.263725550153175</v>
+        <v>0.518883039694389</v>
       </c>
       <c r="C17">
-        <v>-2.43557473627983e-05</v>
+        <v>-3.86949219059067e-05</v>
       </c>
       <c r="D17">
-        <v>6.40324183872774e-06</v>
+        <v>-7.93593270438056e-06</v>
       </c>
       <c r="E17">
-        <v>0.000253404889787946</v>
+        <v>0.000267744064331055</v>
       </c>
       <c r="F17">
-        <v>2.43557473627983e-05</v>
+        <v>3.86949219059067e-05</v>
       </c>
       <c r="G17">
         <v>3.07589892015261e-05</v>
@@ -650,7 +650,7 @@
         <v>0.000229049142425148</v>
       </c>
       <c r="I17">
-        <v>-6.40324183872774e-06</v>
+        <v>7.93593270438056e-06</v>
       </c>
       <c r="J17">
         <v>-3.07589892015261e-05</v>
@@ -666,19 +666,19 @@
         </is>
       </c>
       <c r="B18">
-        <v>4.49495995979987e-10</v>
+        <v>1.10983444656654e-11</v>
       </c>
       <c r="C18">
-        <v>-0.00229637955739495</v>
+        <v>-0.0022701875734908</v>
       </c>
       <c r="D18">
-        <v>-0.00167570795331682</v>
+        <v>-0.00164951596941267</v>
       </c>
       <c r="E18">
-        <v>0.0031698431287493</v>
+        <v>0.00314365114484515</v>
       </c>
       <c r="F18">
-        <v>0.00229637955739495</v>
+        <v>0.0022701875734908</v>
       </c>
       <c r="G18">
         <v>0.00062067160407813</v>
@@ -687,7 +687,7 @@
         <v>0.000873463571354348</v>
       </c>
       <c r="I18">
-        <v>0.00167570795331682</v>
+        <v>0.00164951596941267</v>
       </c>
       <c r="J18">
         <v>-0.00062067160407813</v>
@@ -703,19 +703,19 @@
         </is>
       </c>
       <c r="B19">
-        <v>4.44774772567769e-10</v>
+        <v>2.9339186635724e-10</v>
       </c>
       <c r="C19">
-        <v>0.0007365474702965</v>
+        <v>0.000738216400350211</v>
       </c>
       <c r="D19">
-        <v>0.00144144466945103</v>
+        <v>0.00144311359950474</v>
       </c>
       <c r="E19">
-        <v>0.000140258244105748</v>
+        <v>0.000138589314052037</v>
       </c>
       <c r="F19">
-        <v>-0.0007365474702965</v>
+        <v>-0.000738216400350211</v>
       </c>
       <c r="G19">
         <v>0.000704897199154532</v>
@@ -724,7 +724,7 @@
         <v>0.000876805714402248</v>
       </c>
       <c r="I19">
-        <v>-0.00144144466945103</v>
+        <v>-0.00144311359950474</v>
       </c>
       <c r="J19">
         <v>-0.000704897199154532</v>
@@ -740,19 +740,19 @@
         </is>
       </c>
       <c r="B20">
-        <v>2.43814601841308e-09</v>
+        <v>1.30535515729946e-09</v>
       </c>
       <c r="C20">
-        <v>0.000588332751379182</v>
+        <v>0.000574708832573378</v>
       </c>
       <c r="D20">
-        <v>0.000918660845075334</v>
+        <v>0.00090503692626953</v>
       </c>
       <c r="E20">
-        <v>0.00016157967703683</v>
+        <v>0.000175203595842634</v>
       </c>
       <c r="F20">
-        <v>-0.000588332751379182</v>
+        <v>-0.000574708832573378</v>
       </c>
       <c r="G20">
         <v>0.000330328093696152</v>
@@ -761,7 +761,7 @@
         <v>0.000749912428416012</v>
       </c>
       <c r="I20">
-        <v>-0.000918660845075334</v>
+        <v>-0.00090503692626953</v>
       </c>
       <c r="J20">
         <v>-0.000330328093696152</v>
@@ -777,19 +777,19 @@
         </is>
       </c>
       <c r="B21">
-        <v>2.07276775743281e-08</v>
+        <v>2.80839811406253e-08</v>
       </c>
       <c r="C21">
-        <v>0.000528763915748901</v>
+        <v>0.000516298030041591</v>
       </c>
       <c r="D21">
-        <v>0.000780718667166573</v>
+        <v>0.000768252781459263</v>
       </c>
       <c r="E21">
-        <v>0.000175237655639649</v>
+        <v>0.000187703541346959</v>
       </c>
       <c r="F21">
-        <v>-0.000528763915748901</v>
+        <v>-0.000516298030041591</v>
       </c>
       <c r="G21">
         <v>0.000251954751417673</v>
@@ -798,7 +798,7 @@
         <v>0.000704001571388549</v>
       </c>
       <c r="I21">
-        <v>-0.000780718667166573</v>
+        <v>-0.000768252781459263</v>
       </c>
       <c r="J21">
         <v>-0.000251954751417673</v>
@@ -814,19 +814,19 @@
         </is>
       </c>
       <c r="B22">
-        <v>5.51623191569206e-11</v>
+        <v>3.86991549916615e-11</v>
       </c>
       <c r="C22">
-        <v>-0.00850368647817439</v>
+        <v>-0.00882115784614664</v>
       </c>
       <c r="D22">
-        <v>-0.00876692363194057</v>
+        <v>-0.00908439499991282</v>
       </c>
       <c r="E22">
-        <v>0.00946157319205147</v>
+        <v>0.00977904456002373</v>
       </c>
       <c r="F22">
-        <v>0.00850368647817439</v>
+        <v>0.00882115784614664</v>
       </c>
       <c r="G22">
         <v>-0.000263237153766178</v>
@@ -835,7 +835,7 @@
         <v>0.000957886713877087</v>
       </c>
       <c r="I22">
-        <v>0.00876692363194057</v>
+        <v>0.00908439499991282</v>
       </c>
       <c r="J22">
         <v>0.000263237153766178</v>
@@ -851,19 +851,19 @@
         </is>
       </c>
       <c r="B23">
-        <v>2.80238744432282e-08</v>
+        <v>4.62348825891468e-10</v>
       </c>
       <c r="C23">
-        <v>-0.00913964033783746</v>
+        <v>-0.00930772543610406</v>
       </c>
       <c r="D23">
-        <v>-0.00710402216230119</v>
+        <v>-0.0072721072605678</v>
       </c>
       <c r="E23">
-        <v>0.00945465905325753</v>
+        <v>0.00962274415152413</v>
       </c>
       <c r="F23">
-        <v>0.00913964033783746</v>
+        <v>0.00930772543610406</v>
       </c>
       <c r="G23">
         <v>0.00203561817553626</v>
@@ -872,7 +872,7 @@
         <v>0.000315018715420073</v>
       </c>
       <c r="I23">
-        <v>0.00710402216230119</v>
+        <v>0.0072721072605678</v>
       </c>
       <c r="J23">
         <v>-0.00203561817553626</v>
@@ -888,19 +888,19 @@
         </is>
       </c>
       <c r="B24">
-        <v>1.81178766434087e-08</v>
+        <v>6.80875256175995e-09</v>
       </c>
       <c r="C24">
-        <v>-0.0136215689287513</v>
+        <v>-0.0144235068494579</v>
       </c>
       <c r="D24">
-        <v>-0.0151292255946568</v>
+        <v>-0.0159311635153634</v>
       </c>
       <c r="E24">
-        <v>0.0159100805010114</v>
+        <v>0.0167120184217181</v>
       </c>
       <c r="F24">
-        <v>0.0136215689287513</v>
+        <v>0.0144235068494579</v>
       </c>
       <c r="G24">
         <v>-0.00150765666590554</v>
@@ -909,7 +909,7 @@
         <v>0.00228851157226018</v>
       </c>
       <c r="I24">
-        <v>0.0151292255946568</v>
+        <v>0.0159311635153634</v>
       </c>
       <c r="J24">
         <v>0.00150765666590554</v>
@@ -925,19 +925,19 @@
         </is>
       </c>
       <c r="B25">
-        <v>2.36366741843685e-05</v>
+        <v>7.97397259333366e-10</v>
       </c>
       <c r="C25">
-        <v>-0.000381493577151561</v>
+        <v>-0.000740279478902396</v>
       </c>
       <c r="D25">
-        <v>0.00201940536499023</v>
+        <v>0.0016606194632394</v>
       </c>
       <c r="E25">
-        <v>0.00140469414847238</v>
+        <v>0.00176348005022321</v>
       </c>
       <c r="F25">
-        <v>0.000381493577151561</v>
+        <v>0.000740279478902396</v>
       </c>
       <c r="G25">
         <v>0.00240089894214179</v>
@@ -946,7 +946,7 @@
         <v>0.00102320057132082</v>
       </c>
       <c r="I25">
-        <v>-0.00201940536499023</v>
+        <v>-0.0016606194632394</v>
       </c>
       <c r="J25">
         <v>-0.00240089894214179</v>
@@ -962,19 +962,19 @@
         </is>
       </c>
       <c r="B26">
-        <v>4.00560695723584e-11</v>
+        <v>1.0680345496894e-13</v>
       </c>
       <c r="C26">
-        <v>-0.00730463120791163</v>
+        <v>-0.00750234832958085</v>
       </c>
       <c r="D26">
-        <v>-0.00678181648254394</v>
+        <v>-0.00697953360421317</v>
       </c>
       <c r="E26">
-        <v>0.00776420320783342</v>
+        <v>0.00796192032950265</v>
       </c>
       <c r="F26">
-        <v>0.00730463120791163</v>
+        <v>0.00750234832958085</v>
       </c>
       <c r="G26">
         <v>0.000522814725367685</v>
@@ -983,7 +983,7 @@
         <v>0.000459571999921796</v>
       </c>
       <c r="I26">
-        <v>0.00678181648254394</v>
+        <v>0.00697953360421317</v>
       </c>
       <c r="J26">
         <v>-0.000522814725367685</v>
@@ -999,19 +999,19 @@
         </is>
       </c>
       <c r="B27">
-        <v>5.60720521125546e-08</v>
+        <v>1.84297473948547e-08</v>
       </c>
       <c r="C27">
-        <v>-0.0142123815982943</v>
+        <v>-0.0137640184303954</v>
       </c>
       <c r="D27">
-        <v>-0.0125953810555594</v>
+        <v>-0.0121470178876605</v>
       </c>
       <c r="E27">
-        <v>0.0168675354548863</v>
+        <v>0.0164191722869873</v>
       </c>
       <c r="F27">
-        <v>0.0142123815982943</v>
+        <v>0.0137640184303954</v>
       </c>
       <c r="G27">
         <v>0.00161700054273492</v>
@@ -1020,7 +1020,7 @@
         <v>0.00265515385659195</v>
       </c>
       <c r="I27">
-        <v>0.0125953810555594</v>
+        <v>0.0121470178876605</v>
       </c>
       <c r="J27">
         <v>-0.00161700054273492</v>
@@ -1036,19 +1036,19 @@
         </is>
       </c>
       <c r="B28">
-        <v>0.000204069469053492</v>
+        <v>0.00417047903254708</v>
       </c>
       <c r="C28">
-        <v>0.000360344689397607</v>
+        <v>0.000234766217805113</v>
       </c>
       <c r="D28">
-        <v>9.08715384347095e-05</v>
+        <v>-3.47069331577849e-05</v>
       </c>
       <c r="E28">
-        <v>0.000537463596888951</v>
+        <v>0.000663042068481445</v>
       </c>
       <c r="F28">
-        <v>-0.000360344689397607</v>
+        <v>-0.000234766217805113</v>
       </c>
       <c r="G28">
         <v>-0.000269473150962897</v>
@@ -1057,7 +1057,7 @@
         <v>0.000897808286286558</v>
       </c>
       <c r="I28">
-        <v>-9.08715384347095e-05</v>
+        <v>3.47069331577849e-05</v>
       </c>
       <c r="J28">
         <v>0.000269473150962897</v>
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B29">
-        <v>4.14513379298764e-06</v>
+        <v>6.38050767776122e-07</v>
       </c>
       <c r="C29">
-        <v>-0.0115837598449226</v>
+        <v>-0.00991980252157579</v>
       </c>
       <c r="D29">
-        <v>-0.0100164754050119</v>
+        <v>-0.00835251808166502</v>
       </c>
       <c r="E29">
-        <v>0.0163581371307373</v>
+        <v>0.0146941798073905</v>
       </c>
       <c r="F29">
-        <v>0.0115837598449226</v>
+        <v>0.00991980252157579</v>
       </c>
       <c r="G29">
         <v>0.00156728443991077</v>
@@ -1094,7 +1094,7 @@
         <v>0.00477437728581468</v>
       </c>
       <c r="I29">
-        <v>0.0100164754050119</v>
+        <v>0.00835251808166502</v>
       </c>
       <c r="J29">
         <v>-0.00156728443991077</v>
@@ -1113,16 +1113,16 @@
         <v>0</v>
       </c>
       <c r="C30">
-        <v>0.0243259981803671</v>
+        <v>0.0235695300886748</v>
       </c>
       <c r="D30">
-        <v>-0.00993333544049943</v>
+        <v>-0.0106898035321917</v>
       </c>
       <c r="E30">
-        <v>0.0119738238198416</v>
+        <v>0.0127302919115339</v>
       </c>
       <c r="F30">
-        <v>-0.0243259981803671</v>
+        <v>-0.0235695300886748</v>
       </c>
       <c r="G30">
         <v>-0.0342593336208665</v>
@@ -1131,7 +1131,7 @@
         <v>0.0362998220002087</v>
       </c>
       <c r="I30">
-        <v>0.00993333544049943</v>
+        <v>0.0106898035321917</v>
       </c>
       <c r="J30">
         <v>0.0342593336208665</v>
@@ -1147,19 +1147,19 @@
         </is>
       </c>
       <c r="B31">
-        <v>3.71815900885863e-05</v>
+        <v>8.94061105286559e-05</v>
       </c>
       <c r="C31">
-        <v>-0.00694028859860347</v>
+        <v>-0.00588160792800149</v>
       </c>
       <c r="D31">
-        <v>-0.00919028690883091</v>
+        <v>-0.00813160623822893</v>
       </c>
       <c r="E31">
-        <v>0.0165797301701137</v>
+        <v>0.0155210494995117</v>
       </c>
       <c r="F31">
-        <v>0.00694028859860347</v>
+        <v>0.00588160792800149</v>
       </c>
       <c r="G31">
         <v>-0.00224999831022744</v>
@@ -1168,7 +1168,7 @@
         <v>0.00963944157151023</v>
       </c>
       <c r="I31">
-        <v>0.00919028690883091</v>
+        <v>0.00813160623822893</v>
       </c>
       <c r="J31">
         <v>0.00224999831022744</v>
@@ -1184,19 +1184,19 @@
         </is>
       </c>
       <c r="B32">
-        <v>2.8709572164054e-08</v>
+        <v>2.18244893746e-06</v>
       </c>
       <c r="C32">
-        <v>-0.00407207411938413</v>
+        <v>-0.00381076735668882</v>
       </c>
       <c r="D32">
-        <v>-0.00259365354265485</v>
+        <v>-0.00233234677995954</v>
       </c>
       <c r="E32">
-        <v>0.00651243754795619</v>
+        <v>0.00625113078526088</v>
       </c>
       <c r="F32">
-        <v>0.00407207411938413</v>
+        <v>0.00381076735668882</v>
       </c>
       <c r="G32">
         <v>0.00147842057672928</v>
@@ -1205,7 +1205,7 @@
         <v>0.00244036342857206</v>
       </c>
       <c r="I32">
-        <v>0.00259365354265485</v>
+        <v>0.00233234677995954</v>
       </c>
       <c r="J32">
         <v>-0.00147842057672928</v>
@@ -1221,19 +1221,19 @@
         </is>
       </c>
       <c r="B33">
-        <v>3.99673611983786e-07</v>
+        <v>1.00862142227154e-06</v>
       </c>
       <c r="C33">
-        <v>-0.00185010132138684</v>
+        <v>-0.00170790166885126</v>
       </c>
       <c r="D33">
-        <v>-0.00233939715794155</v>
+        <v>-0.00219719750540597</v>
       </c>
       <c r="E33">
-        <v>0.00410066332135882</v>
+        <v>0.00395846366882324</v>
       </c>
       <c r="F33">
-        <v>0.00185010132138684</v>
+        <v>0.00170790166885126</v>
       </c>
       <c r="G33">
         <v>-0.000489295836554707</v>
@@ -1242,7 +1242,7 @@
         <v>0.00225056199997198</v>
       </c>
       <c r="I33">
-        <v>0.00233939715794155</v>
+        <v>0.00219719750540597</v>
       </c>
       <c r="J33">
         <v>0.000489295836554707</v>

</xml_diff>